<commit_message>
rozpoczęcie pracy nad Sprawodzaniem
</commit_message>
<xml_diff>
--- a/wykresy.xlsx
+++ b/wykresy.xlsx
@@ -8,22 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sansrozpierducha/Programy/P02_Mateusz_Dzialowski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F430C1D6-5204-8F4A-9C3C-DA3A84EC14FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E9C76BA-AAE8-D149-B727-2AF432D10AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20420" yWindow="3780" windowWidth="30480" windowHeight="20200" xr2:uid="{534139F7-C274-0A41-B767-3A8E13DF0B1C}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19760" xr2:uid="{534139F7-C274-0A41-B767-3A8E13DF0B1C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$B$1</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$B$2:$B$11</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Sheet1!$D$1</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Sheet1!$D$2:$D$11</definedName>
-    <definedName name="_xlchart.v2.0" hidden="1">Sheet1!$B$1</definedName>
-    <definedName name="_xlchart.v2.1" hidden="1">Sheet1!$B$2:$B$11</definedName>
-    <definedName name="_xlchart.v2.2" hidden="1">Sheet1!$D$1</definedName>
-    <definedName name="_xlchart.v2.3" hidden="1">Sheet1!$D$2:$D$11</definedName>
     <definedName name="wyniki_wydajnosci" localSheetId="0">Sheet1!$A$1:$D$11</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
@@ -49,7 +41,7 @@
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
 <connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
   <connection id="1" xr16:uid="{4BB6F3F9-809A-D149-923C-EB07D6DA4651}" name="wyniki_wydajnosci" type="6" refreshedVersion="8" background="1" saveData="1">
-    <textPr codePage="10000" sourceFile="/Users/sansrozpierducha/Programy/P02_Mateusz_Dzialowski/wyniki_wydajnosci.txt" thousands=" " tab="0" space="1" consecutive="1">
+    <textPr sourceFile="/Users/sansrozpierducha/Programy/P02_Mateusz_Dzialowski/wyniki_wydajnosci.txt" thousands=" " tab="0" space="1" consecutive="1">
       <textFields count="4">
         <textField/>
         <textField/>
@@ -533,7 +525,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.13667146873074476"/>
+          <c:y val="0.17171296296296296"/>
+          <c:w val="0.80716471645743104"/>
+          <c:h val="0.73278178769320501"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
@@ -797,7 +799,7 @@
         <c:crossAx val="1828389311"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
-        <c:minorUnit val="1.0000000000000001E-5"/>
+        <c:minorUnit val="1E-4"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -1997,13 +1999,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
+      <xdr:colOff>209549</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>8467</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>658283</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>296332</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>110067</xdr:rowOff>
     </xdr:to>

</xml_diff>